<commit_message>
- Updated the configuration file
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Config\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFBA958-8818-4E40-8714-676C47D5BFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15375" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,53 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Data\Input\Daily_Transactions.xlsx</t>
+  </si>
+  <si>
+    <t>C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Data\Input\Suspicious_Accounts.csv</t>
+  </si>
+  <si>
+    <t>C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Data\Output\Reports</t>
+  </si>
+  <si>
+    <t>Output_Reports_Folder</t>
+  </si>
+  <si>
+    <t>Daily_Transactions_Path</t>
+  </si>
+  <si>
+    <t>Suspicious_Accounts_Path</t>
+  </si>
+  <si>
+    <t>C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Data\Templates</t>
+  </si>
+  <si>
+    <t>Transaction_Report_Template</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +380,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="78.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
- Moved data from dtConfigTable to a dictionary called dictConfigLocal - Looped dictionary and printed its data - Added two new variable to the config.xlsx file (Thresh_Hold_Amount,Risky_Transaction_Type)
</commit_message>
<xml_diff>
--- a/Config/Config.xlsx
+++ b/Config/Config.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFBA958-8818-4E40-8714-676C47D5BFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E7B250-B766-4B1D-9B5A-92F9BD85FFAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15375" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2190" yWindow="3570" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Key</t>
   </si>
@@ -45,16 +45,25 @@
     <t>Output_Reports_Folder</t>
   </si>
   <si>
-    <t>Daily_Transactions_Path</t>
-  </si>
-  <si>
-    <t>Suspicious_Accounts_Path</t>
-  </si>
-  <si>
     <t>C:\Users\BloodB\Documents\UiPath\PM-04-PS07\Data\Templates</t>
   </si>
   <si>
     <t>Transaction_Report_Template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Daily_Transactions_Path   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suspicious_Accounts_Path </t>
+  </si>
+  <si>
+    <t>Thresh_Hold_Amount</t>
+  </si>
+  <si>
+    <t>Risky_Transaction_Type</t>
+  </si>
+  <si>
+    <t>International</t>
   </si>
 </sst>
 </file>
@@ -381,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
@@ -398,7 +407,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -406,7 +415,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -422,10 +431,26 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>